<commit_message>
Save owner approval of Hisnul Muslim entries 78 through 261
</commit_message>
<xml_diff>
--- a/training-data/reusable-language-memory/hisnul-muslim/Hisnul-Muslim-Kashmiri-Review-v2.xlsx
+++ b/training-data/reusable-language-memory/hisnul-muslim/Hisnul-Muslim-Kashmiri-Review-v2.xlsx
@@ -6073,10 +6073,14 @@
       <c r="I79" s="8" t="inlineStr"/>
       <c r="J79" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K79" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K79" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L79" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6131,10 +6135,14 @@
       <c r="I80" s="8" t="inlineStr"/>
       <c r="J80" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K80" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K80" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6186,10 +6194,14 @@
       <c r="I81" s="8" t="inlineStr"/>
       <c r="J81" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K81" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K81" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L81" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6241,10 +6253,14 @@
       <c r="I82" s="8" t="inlineStr"/>
       <c r="J82" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K82" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K82" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6296,10 +6312,14 @@
       <c r="I83" s="8" t="inlineStr"/>
       <c r="J83" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K83" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K83" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L83" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6347,10 +6367,14 @@
       <c r="I84" s="8" t="inlineStr"/>
       <c r="J84" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K84" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K84" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6398,10 +6422,14 @@
       <c r="I85" s="8" t="inlineStr"/>
       <c r="J85" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K85" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K85" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L85" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6453,10 +6481,14 @@
       <c r="I86" s="8" t="inlineStr"/>
       <c r="J86" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K86" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K86" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6508,10 +6540,14 @@
       <c r="I87" s="8" t="inlineStr"/>
       <c r="J87" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K87" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K87" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L87" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6563,10 +6599,14 @@
       <c r="I88" s="8" t="inlineStr"/>
       <c r="J88" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K88" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K88" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6618,10 +6658,14 @@
       <c r="I89" s="8" t="inlineStr"/>
       <c r="J89" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K89" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K89" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L89" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6669,10 +6713,14 @@
       <c r="I90" s="8" t="inlineStr"/>
       <c r="J90" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K90" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K90" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L90" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6724,10 +6772,14 @@
       <c r="I91" s="8" t="inlineStr"/>
       <c r="J91" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K91" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K91" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L91" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6776,10 +6828,14 @@
       <c r="I92" s="8" t="inlineStr"/>
       <c r="J92" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K92" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K92" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L92" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6831,10 +6887,14 @@
       <c r="I93" s="8" t="inlineStr"/>
       <c r="J93" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K93" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K93" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L93" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6889,10 +6949,14 @@
       <c r="I94" s="8" t="inlineStr"/>
       <c r="J94" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K94" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K94" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L94" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -6946,10 +7010,14 @@
       <c r="I95" s="8" t="inlineStr"/>
       <c r="J95" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K95" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K95" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L95" s="5" t="inlineStr">
         <is>
           <t>The three surahs are expanded from the comparison text; also reproduced on Quran Passages sheet.</t>
@@ -7001,10 +7069,14 @@
       <c r="I96" s="8" t="inlineStr"/>
       <c r="J96" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K96" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K96" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L96" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7056,10 +7128,14 @@
       <c r="I97" s="8" t="inlineStr"/>
       <c r="J97" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K97" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K97" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L97" s="5" t="inlineStr">
         <is>
           <t>Ayat al-Kursi expanded from the comparison text; PDF references the verse.</t>
@@ -7112,10 +7188,14 @@
       <c r="I98" s="8" t="inlineStr"/>
       <c r="J98" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K98" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K98" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
           <t>Quran 2:285–286 expanded for review; PDF references these verses.</t>
@@ -7167,10 +7247,14 @@
       <c r="I99" s="8" t="inlineStr"/>
       <c r="J99" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K99" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K99" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L99" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7218,10 +7302,14 @@
       <c r="I100" s="8" t="inlineStr"/>
       <c r="J100" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K100" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K100" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7273,10 +7361,14 @@
       <c r="I101" s="8" t="inlineStr"/>
       <c r="J101" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K101" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K101" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L101" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7324,10 +7416,14 @@
       <c r="I102" s="8" t="inlineStr"/>
       <c r="J102" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K102" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K102" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7379,10 +7475,14 @@
       <c r="I103" s="8" t="inlineStr"/>
       <c r="J103" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K103" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K103" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L103" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7434,10 +7534,14 @@
       <c r="I104" s="8" t="inlineStr"/>
       <c r="J104" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K104" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K104" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
           <t>Review divine names az-Zahir/al-Batin; translation is a draft, not a doctrinal ruling.</t>
@@ -7485,10 +7589,14 @@
       <c r="I105" s="8" t="inlineStr"/>
       <c r="J105" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K105" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K105" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L105" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7536,10 +7644,14 @@
       <c r="I106" s="8" t="inlineStr"/>
       <c r="J106" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K106" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K106" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L106" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7591,10 +7703,14 @@
       <c r="I107" s="8" t="inlineStr"/>
       <c r="J107" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K107" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K107" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L107" s="5" t="inlineStr">
         <is>
           <t>PDF instructs recitation of Surahs 32 and 67; it does not print the full chapters. The instruction, not the full chapters, is translated.</t>
@@ -7646,10 +7762,14 @@
       <c r="I108" s="8" t="inlineStr"/>
       <c r="J108" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K108" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K108" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L108" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7697,10 +7817,14 @@
       <c r="I109" s="8" t="inlineStr"/>
       <c r="J109" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K109" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K109" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L109" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7748,10 +7872,14 @@
       <c r="I110" s="8" t="inlineStr"/>
       <c r="J110" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K110" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K110" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7803,10 +7931,14 @@
       <c r="I111" s="8" t="inlineStr"/>
       <c r="J111" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K111" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K111" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L111" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7854,10 +7986,14 @@
       <c r="I112" s="8" t="inlineStr"/>
       <c r="J112" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K112" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K112" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -7905,10 +8041,14 @@
       <c r="I113" s="8" t="inlineStr"/>
       <c r="J113" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K113" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K113" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L113" s="5" t="inlineStr">
         <is>
           <t>Review rendering of the decree clause in Witr qunut.</t>
@@ -7956,10 +8096,14 @@
       <c r="I114" s="8" t="inlineStr"/>
       <c r="J114" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K114" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K114" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L114" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8007,10 +8151,14 @@
       <c r="I115" s="8" t="inlineStr"/>
       <c r="J115" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K115" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K115" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L115" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8062,10 +8210,14 @@
       <c r="I116" s="8" t="inlineStr"/>
       <c r="J116" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K116" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K116" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8113,10 +8265,14 @@
       <c r="I117" s="8" t="inlineStr"/>
       <c r="J117" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K117" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K117" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L117" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8164,10 +8320,14 @@
       <c r="I118" s="8" t="inlineStr"/>
       <c r="J118" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K118" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K118" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L118" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8215,10 +8375,14 @@
       <c r="I119" s="8" t="inlineStr"/>
       <c r="J119" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K119" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K119" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L119" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8266,10 +8430,14 @@
       <c r="I120" s="8" t="inlineStr"/>
       <c r="J120" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K120" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K120" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L120" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8317,10 +8485,14 @@
       <c r="I121" s="8" t="inlineStr"/>
       <c r="J121" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K121" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K121" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L121" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8368,10 +8540,14 @@
       <c r="I122" s="8" t="inlineStr"/>
       <c r="J122" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K122" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K122" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L122" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8419,10 +8595,14 @@
       <c r="I123" s="8" t="inlineStr"/>
       <c r="J123" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K123" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K123" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L123" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8470,10 +8650,14 @@
       <c r="I124" s="8" t="inlineStr"/>
       <c r="J124" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K124" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K124" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L124" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8521,10 +8705,14 @@
       <c r="I125" s="8" t="inlineStr"/>
       <c r="J125" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K125" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K125" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L125" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8576,10 +8764,14 @@
       <c r="I126" s="8" t="inlineStr"/>
       <c r="J126" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K126" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K126" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L126" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8627,10 +8819,14 @@
       <c r="I127" s="8" t="inlineStr"/>
       <c r="J127" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K127" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K127" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L127" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8682,10 +8878,14 @@
       <c r="I128" s="8" t="inlineStr"/>
       <c r="J128" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K128" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K128" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L128" s="3" t="inlineStr">
         <is>
           <t>Quran 57:3; review divine names az-Zahir/al-Batin.</t>
@@ -8733,10 +8933,14 @@
       <c r="I129" s="8" t="inlineStr"/>
       <c r="J129" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K129" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K129" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L129" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8784,10 +8988,14 @@
       <c r="I130" s="8" t="inlineStr"/>
       <c r="J130" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K130" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K130" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L130" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8839,10 +9047,14 @@
       <c r="I131" s="8" t="inlineStr"/>
       <c r="J131" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K131" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K131" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L131" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8890,10 +9102,14 @@
       <c r="I132" s="8" t="inlineStr"/>
       <c r="J132" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K132" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K132" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L132" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8941,10 +9157,14 @@
       <c r="I133" s="8" t="inlineStr"/>
       <c r="J133" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K133" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K133" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L133" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -8992,10 +9212,14 @@
       <c r="I134" s="8" t="inlineStr"/>
       <c r="J134" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K134" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K134" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L134" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9043,10 +9267,14 @@
       <c r="I135" s="8" t="inlineStr"/>
       <c r="J135" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K135" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K135" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L135" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9094,10 +9322,14 @@
       <c r="I136" s="8" t="inlineStr"/>
       <c r="J136" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K136" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K136" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L136" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9145,10 +9377,14 @@
       <c r="I137" s="8" t="inlineStr"/>
       <c r="J137" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K137" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K137" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L137" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9200,10 +9436,14 @@
       <c r="I138" s="8" t="inlineStr"/>
       <c r="J138" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K138" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K138" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L138" s="3" t="inlineStr">
         <is>
           <t>Distinct from the other edition: PDF #137 is hasbi Allah wa nim al-wakil, NOT congratulations for a newborn.</t>
@@ -9255,10 +9495,14 @@
       <c r="I139" s="8" t="inlineStr"/>
       <c r="J139" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K139" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K139" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L139" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9306,10 +9550,14 @@
       <c r="I140" s="8" t="inlineStr"/>
       <c r="J140" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K140" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K140" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L140" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9361,10 +9609,14 @@
       <c r="I141" s="8" t="inlineStr"/>
       <c r="J141" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K141" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K141" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L141" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9412,10 +9664,14 @@
       <c r="I142" s="8" t="inlineStr"/>
       <c r="J142" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K142" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K142" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L142" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9463,10 +9719,14 @@
       <c r="I143" s="8" t="inlineStr"/>
       <c r="J143" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K143" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K143" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L143" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9518,10 +9778,14 @@
       <c r="I144" s="8" t="inlineStr"/>
       <c r="J144" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K144" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K144" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L144" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9569,10 +9833,14 @@
       <c r="I145" s="8" t="inlineStr"/>
       <c r="J145" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K145" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K145" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L145" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9624,10 +9892,14 @@
       <c r="I146" s="8" t="inlineStr"/>
       <c r="J146" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K146" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K146" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9675,10 +9947,14 @@
       <c r="I147" s="8" t="inlineStr"/>
       <c r="J147" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K147" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K147" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L147" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9726,10 +10002,14 @@
       <c r="I148" s="8" t="inlineStr"/>
       <c r="J148" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K148" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K148" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L148" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9781,10 +10061,14 @@
       <c r="I149" s="8" t="inlineStr"/>
       <c r="J149" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K149" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K149" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L149" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9832,10 +10116,14 @@
       <c r="I150" s="8" t="inlineStr"/>
       <c r="J150" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K150" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K150" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L150" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9887,10 +10175,14 @@
       <c r="I151" s="8" t="inlineStr"/>
       <c r="J151" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K151" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K151" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L151" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9938,10 +10230,14 @@
       <c r="I152" s="8" t="inlineStr"/>
       <c r="J152" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K152" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K152" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L152" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -9993,10 +10289,14 @@
       <c r="I153" s="8" t="inlineStr"/>
       <c r="J153" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K153" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K153" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L153" s="5" t="inlineStr">
         <is>
           <t>PDF child-funeral wording used; extra clauses in the comparison edition were excluded.</t>
@@ -10044,10 +10344,14 @@
       <c r="I154" s="8" t="inlineStr"/>
       <c r="J154" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K154" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K154" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L154" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10099,10 +10403,14 @@
       <c r="I155" s="8" t="inlineStr"/>
       <c r="J155" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K155" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K155" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L155" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10150,10 +10458,14 @@
       <c r="I156" s="8" t="inlineStr"/>
       <c r="J156" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K156" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K156" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L156" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10205,10 +10517,14 @@
       <c r="I157" s="8" t="inlineStr"/>
       <c r="J157" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K157" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K157" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L157" s="5" t="inlineStr">
         <is>
           <t>PDF is a narration instructing dua, not a fixed quoted formula; translation preserves the instruction.</t>
@@ -10256,10 +10572,14 @@
       <c r="I158" s="8" t="inlineStr"/>
       <c r="J158" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K158" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K158" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L158" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10307,10 +10627,14 @@
       <c r="I159" s="8" t="inlineStr"/>
       <c r="J159" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K159" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K159" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L159" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10358,10 +10682,14 @@
       <c r="I160" s="8" t="inlineStr"/>
       <c r="J160" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K160" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K160" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L160" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10413,10 +10741,14 @@
       <c r="I161" s="8" t="inlineStr"/>
       <c r="J161" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K161" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K161" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L161" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10464,10 +10796,14 @@
       <c r="I162" s="8" t="inlineStr"/>
       <c r="J162" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K162" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K162" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L162" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10515,10 +10851,14 @@
       <c r="I163" s="8" t="inlineStr"/>
       <c r="J163" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K163" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K163" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L163" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10566,10 +10906,14 @@
       <c r="I164" s="8" t="inlineStr"/>
       <c r="J164" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K164" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K164" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L164" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10617,10 +10961,14 @@
       <c r="I165" s="8" t="inlineStr"/>
       <c r="J165" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K165" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K165" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L165" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10668,10 +11016,14 @@
       <c r="I166" s="8" t="inlineStr"/>
       <c r="J166" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K166" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K166" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L166" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10719,10 +11071,14 @@
       <c r="I167" s="8" t="inlineStr"/>
       <c r="J167" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K167" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K167" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L167" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10774,10 +11130,14 @@
       <c r="I168" s="8" t="inlineStr"/>
       <c r="J168" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K168" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K168" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L168" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10829,10 +11189,14 @@
       <c r="I169" s="8" t="inlineStr"/>
       <c r="J169" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K169" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K169" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L169" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10884,10 +11248,14 @@
       <c r="I170" s="8" t="inlineStr"/>
       <c r="J170" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K170" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K170" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L170" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10935,10 +11303,14 @@
       <c r="I171" s="8" t="inlineStr"/>
       <c r="J171" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K171" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K171" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L171" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -10987,10 +11359,14 @@
       <c r="I172" s="8" t="inlineStr"/>
       <c r="J172" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K172" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K172" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L172" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11038,10 +11414,14 @@
       <c r="I173" s="8" t="inlineStr"/>
       <c r="J173" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K173" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K173" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L173" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11093,10 +11473,14 @@
       <c r="I174" s="8" t="inlineStr"/>
       <c r="J174" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K174" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K174" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L174" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11144,10 +11528,14 @@
       <c r="I175" s="8" t="inlineStr"/>
       <c r="J175" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K175" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K175" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L175" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11195,10 +11583,14 @@
       <c r="I176" s="8" t="inlineStr"/>
       <c r="J176" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K176" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K176" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L176" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11246,10 +11638,14 @@
       <c r="I177" s="8" t="inlineStr"/>
       <c r="J177" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K177" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K177" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L177" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11301,10 +11697,14 @@
       <c r="I178" s="8" t="inlineStr"/>
       <c r="J178" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K178" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K178" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L178" s="3" t="inlineStr">
         <is>
           <t>Comparison English erroneously says not invited; Arabic/PDF say if invited. Corrected in draft.</t>
@@ -11356,10 +11756,14 @@
       <c r="I179" s="8" t="inlineStr"/>
       <c r="J179" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K179" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K179" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L179" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11411,10 +11815,14 @@
       <c r="I180" s="8" t="inlineStr"/>
       <c r="J180" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K180" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K180" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L180" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11462,10 +11870,14 @@
       <c r="I181" s="8" t="inlineStr"/>
       <c r="J181" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K181" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K181" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L181" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11517,10 +11929,14 @@
       <c r="I182" s="8" t="inlineStr"/>
       <c r="J182" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K182" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K182" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L182" s="3" t="inlineStr">
         <is>
           <t>Review gender/context: spouse and historical animal-purchase setting.</t>
@@ -11568,10 +11984,14 @@
       <c r="I183" s="8" t="inlineStr"/>
       <c r="J183" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K183" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K183" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L183" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11619,10 +12039,14 @@
       <c r="I184" s="8" t="inlineStr"/>
       <c r="J184" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K184" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K184" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L184" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11670,10 +12094,14 @@
       <c r="I185" s="8" t="inlineStr"/>
       <c r="J185" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K185" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K185" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L185" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11725,10 +12153,14 @@
       <c r="I186" s="8" t="inlineStr"/>
       <c r="J186" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K186" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K186" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L186" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11776,10 +12208,14 @@
       <c r="I187" s="8" t="inlineStr"/>
       <c r="J187" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K187" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K187" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L187" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11831,10 +12267,14 @@
       <c r="I188" s="8" t="inlineStr"/>
       <c r="J188" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K188" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K188" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L188" s="3" t="inlineStr">
         <is>
           <t>Repeated closing dhikr preserved as its own PDF entry; PDF wording omits Allahumma.</t>
@@ -11882,10 +12322,14 @@
       <c r="I189" s="8" t="inlineStr"/>
       <c r="J189" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K189" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K189" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L189" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11933,10 +12377,14 @@
       <c r="I190" s="8" t="inlineStr"/>
       <c r="J190" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K190" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K190" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L190" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -11988,10 +12436,14 @@
       <c r="I191" s="8" t="inlineStr"/>
       <c r="J191" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K191" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K191" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L191" s="5" t="inlineStr">
         <is>
           <t>PDF references ten opening verses of al-Kahf; the book does not print the full passage. Instructions translated.</t>
@@ -12039,10 +12491,14 @@
       <c r="I192" s="8" t="inlineStr"/>
       <c r="J192" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K192" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K192" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L192" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12090,10 +12546,14 @@
       <c r="I193" s="8" t="inlineStr"/>
       <c r="J193" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K193" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K193" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L193" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12141,10 +12601,14 @@
       <c r="I194" s="8" t="inlineStr"/>
       <c r="J194" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K194" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K194" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L194" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12192,10 +12656,14 @@
       <c r="I195" s="8" t="inlineStr"/>
       <c r="J195" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K195" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K195" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L195" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12247,10 +12715,14 @@
       <c r="I196" s="8" t="inlineStr"/>
       <c r="J196" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K196" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K196" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L196" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12298,10 +12770,14 @@
       <c r="I197" s="8" t="inlineStr"/>
       <c r="J197" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K197" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K197" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L197" s="5" t="inlineStr">
         <is>
           <t>Bad-omen wording is a meaning-based rendering; reviewer should verify phrase la tayra illa tayruk.</t>
@@ -12353,10 +12829,14 @@
       <c r="I198" s="8" t="inlineStr"/>
       <c r="J198" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K198" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K198" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L198" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12409,10 +12889,14 @@
       <c r="I199" s="8" t="inlineStr"/>
       <c r="J199" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K199" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K199" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L199" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12460,10 +12944,14 @@
       <c r="I200" s="8" t="inlineStr"/>
       <c r="J200" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K200" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K200" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L200" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12511,10 +12999,14 @@
       <c r="I201" s="8" t="inlineStr"/>
       <c r="J201" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K201" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K201" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L201" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12562,10 +13054,14 @@
       <c r="I202" s="8" t="inlineStr"/>
       <c r="J202" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K202" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K202" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L202" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12613,10 +13109,14 @@
       <c r="I203" s="8" t="inlineStr"/>
       <c r="J203" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K203" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K203" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L203" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12664,10 +13164,14 @@
       <c r="I204" s="8" t="inlineStr"/>
       <c r="J204" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K204" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K204" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L204" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12715,10 +13219,14 @@
       <c r="I205" s="8" t="inlineStr"/>
       <c r="J205" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K205" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K205" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L205" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12770,10 +13278,14 @@
       <c r="I206" s="8" t="inlineStr"/>
       <c r="J206" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K206" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K206" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L206" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12821,10 +13333,14 @@
       <c r="I207" s="8" t="inlineStr"/>
       <c r="J207" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K207" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K207" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L207" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12872,10 +13388,14 @@
       <c r="I208" s="8" t="inlineStr"/>
       <c r="J208" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K208" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K208" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L208" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12927,10 +13447,14 @@
       <c r="I209" s="8" t="inlineStr"/>
       <c r="J209" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K209" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K209" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L209" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -12978,10 +13502,14 @@
       <c r="I210" s="8" t="inlineStr"/>
       <c r="J210" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K210" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K210" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L210" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13033,10 +13561,14 @@
       <c r="I211" s="8" t="inlineStr"/>
       <c r="J211" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K211" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K211" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L211" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13084,10 +13616,14 @@
       <c r="I212" s="8" t="inlineStr"/>
       <c r="J212" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K212" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K212" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L212" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13135,10 +13671,14 @@
       <c r="I213" s="8" t="inlineStr"/>
       <c r="J213" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K213" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K213" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L213" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13186,10 +13726,14 @@
       <c r="I214" s="8" t="inlineStr"/>
       <c r="J214" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K214" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K214" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L214" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13237,10 +13781,14 @@
       <c r="I215" s="8" t="inlineStr"/>
       <c r="J215" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K215" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K215" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L215" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13288,10 +13836,14 @@
       <c r="I216" s="8" t="inlineStr"/>
       <c r="J216" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K216" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K216" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L216" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13339,10 +13891,14 @@
       <c r="I217" s="8" t="inlineStr"/>
       <c r="J217" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K217" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K217" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L217" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13390,10 +13946,14 @@
       <c r="I218" s="8" t="inlineStr"/>
       <c r="J218" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K218" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K218" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L218" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13441,10 +14001,14 @@
       <c r="I219" s="8" t="inlineStr"/>
       <c r="J219" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K219" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K219" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L219" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13492,10 +14056,14 @@
       <c r="I220" s="8" t="inlineStr"/>
       <c r="J220" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K220" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K220" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L220" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13543,10 +14111,14 @@
       <c r="I221" s="8" t="inlineStr"/>
       <c r="J221" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K221" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K221" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L221" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13599,10 +14171,14 @@
       <c r="I222" s="8" t="inlineStr"/>
       <c r="J222" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K222" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K222" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L222" s="3" t="inlineStr">
         <is>
           <t>PDF includes Quran 2:158 excerpt, dhikr and ritual directions; keep them distinct.</t>
@@ -13654,10 +14230,14 @@
       <c r="I223" s="8" t="inlineStr"/>
       <c r="J223" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K223" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K223" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L223" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13705,10 +14285,14 @@
       <c r="I224" s="8" t="inlineStr"/>
       <c r="J224" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K224" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K224" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L224" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13756,10 +14340,14 @@
       <c r="I225" s="8" t="inlineStr"/>
       <c r="J225" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K225" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K225" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L225" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13811,10 +14399,14 @@
       <c r="I226" s="8" t="inlineStr"/>
       <c r="J226" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K226" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K226" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L226" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13862,10 +14454,14 @@
       <c r="I227" s="8" t="inlineStr"/>
       <c r="J227" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K227" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K227" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L227" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13913,10 +14509,14 @@
       <c r="I228" s="8" t="inlineStr"/>
       <c r="J228" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K228" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K228" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L228" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -13964,10 +14564,14 @@
       <c r="I229" s="8" t="inlineStr"/>
       <c r="J229" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K229" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K229" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L229" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14015,10 +14619,14 @@
       <c r="I230" s="8" t="inlineStr"/>
       <c r="J230" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K230" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K230" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L230" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14066,10 +14674,14 @@
       <c r="I231" s="8" t="inlineStr"/>
       <c r="J231" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K231" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K231" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L231" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14121,10 +14733,14 @@
       <c r="I232" s="8" t="inlineStr"/>
       <c r="J232" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K232" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K232" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L232" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14179,10 +14795,14 @@
       <c r="I233" s="8" t="inlineStr"/>
       <c r="J233" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K233" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K233" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L233" s="5" t="inlineStr">
         <is>
           <t>Both extra supplications in the PDF footnote included, separate from the instruction.</t>
@@ -14230,10 +14850,14 @@
       <c r="I234" s="8" t="inlineStr"/>
       <c r="J234" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K234" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K234" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L234" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14281,10 +14905,14 @@
       <c r="I235" s="8" t="inlineStr"/>
       <c r="J235" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K235" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K235" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L235" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14332,10 +14960,14 @@
       <c r="I236" s="8" t="inlineStr"/>
       <c r="J236" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K236" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K236" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L236" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14383,10 +15015,14 @@
       <c r="I237" s="8" t="inlineStr"/>
       <c r="J237" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K237" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K237" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L237" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14434,10 +15070,14 @@
       <c r="I238" s="8" t="inlineStr"/>
       <c r="J238" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K238" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K238" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L238" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14485,10 +15125,14 @@
       <c r="I239" s="8" t="inlineStr"/>
       <c r="J239" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K239" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K239" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L239" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14540,10 +15184,14 @@
       <c r="I240" s="8" t="inlineStr"/>
       <c r="J240" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K240" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K240" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L240" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14591,10 +15239,14 @@
       <c r="I241" s="8" t="inlineStr"/>
       <c r="J241" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K241" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K241" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L241" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14646,10 +15298,14 @@
       <c r="I242" s="8" t="inlineStr"/>
       <c r="J242" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K242" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K242" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L242" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14701,10 +15357,14 @@
       <c r="I243" s="8" t="inlineStr"/>
       <c r="J243" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K243" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K243" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L243" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14756,10 +15416,14 @@
       <c r="I244" s="8" t="inlineStr"/>
       <c r="J244" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K244" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K244" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L244" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14807,10 +15471,14 @@
       <c r="I245" s="8" t="inlineStr"/>
       <c r="J245" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K245" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K245" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L245" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14858,10 +15526,14 @@
       <c r="I246" s="8" t="inlineStr"/>
       <c r="J246" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K246" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K246" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L246" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -14913,10 +15585,14 @@
       <c r="I247" s="8" t="inlineStr"/>
       <c r="J247" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K247" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K247" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L247" s="5" t="inlineStr">
         <is>
           <t>Review nuanced term yughanu; no claim of prophetic sin is inferred.</t>
@@ -14968,10 +15644,14 @@
       <c r="I248" s="8" t="inlineStr"/>
       <c r="J248" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K248" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K248" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L248" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15023,10 +15703,14 @@
       <c r="I249" s="8" t="inlineStr"/>
       <c r="J249" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K249" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K249" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L249" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15078,10 +15762,14 @@
       <c r="I250" s="8" t="inlineStr"/>
       <c r="J250" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K250" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K250" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L250" s="3" t="inlineStr">
         <is>
           <t>PDF #249 is subhan Allah wa bihamdihi, not the tawhid formula. Mapping corrected after reading page 267.</t>
@@ -15133,10 +15821,14 @@
       <c r="I251" s="8" t="inlineStr"/>
       <c r="J251" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K251" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K251" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L251" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15188,10 +15880,14 @@
       <c r="I252" s="8" t="inlineStr"/>
       <c r="J252" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K252" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K252" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L252" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15243,10 +15939,14 @@
       <c r="I253" s="8" t="inlineStr"/>
       <c r="J253" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K253" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K253" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L253" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15298,10 +15998,14 @@
       <c r="I254" s="8" t="inlineStr"/>
       <c r="J254" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K254" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K254" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L254" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15353,10 +16057,14 @@
       <c r="I255" s="8" t="inlineStr"/>
       <c r="J255" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K255" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K255" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L255" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15408,10 +16116,14 @@
       <c r="I256" s="8" t="inlineStr"/>
       <c r="J256" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K256" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K256" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L256" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15463,10 +16175,14 @@
       <c r="I257" s="8" t="inlineStr"/>
       <c r="J257" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K257" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K257" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L257" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15519,10 +16235,14 @@
       <c r="I258" s="8" t="inlineStr"/>
       <c r="J258" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K258" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K258" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L258" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15574,10 +16294,14 @@
       <c r="I259" s="8" t="inlineStr"/>
       <c r="J259" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K259" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K259" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L259" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15625,10 +16349,14 @@
       <c r="I260" s="8" t="inlineStr"/>
       <c r="J260" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K260" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K260" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L260" s="3" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15676,10 +16404,14 @@
       <c r="I261" s="8" t="inlineStr"/>
       <c r="J261" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K261" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K261" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L261" s="5" t="inlineStr">
         <is>
           <t>Draft: compare Kashmiri meaning, Arabic wording and recitation context against the uploaded PDF.</t>
@@ -15732,10 +16464,14 @@
       <c r="I262" s="8" t="inlineStr"/>
       <c r="J262" s="8" t="inlineStr">
         <is>
-          <t>Awaiting your review</t>
-        </is>
-      </c>
-      <c r="K262" s="8" t="inlineStr"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K262" s="8" t="inlineStr">
+        <is>
+          <t>Owner approved entries 78–261 in the simplified review workbook: All correct. See approved-entries-78-261.json for exact approved text.</t>
+        </is>
+      </c>
       <c r="L262" s="3" t="inlineStr">
         <is>
           <t>Final unnumbered book-closing dua included with the final numbered entry.</t>

</xml_diff>